<commit_message>
- move constants_items into the master data source with tests - fix load_constants so object-shaped constants aren't nested under name__ - load .env from dota2_dbt/ in all ingestion scripts - build seeds into their own schema, create DOTA2_STAGING in setup script
</commit_message>
<xml_diff>
--- a/docs/sttm_raw_to_staging.xlsx
+++ b/docs/sttm_raw_to_staging.xlsx
@@ -3147,10 +3147,14 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>New technical key, not dlt_id itself</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr"/>
+          <t>would carry through as dim_item's key at mart, but dim_item is on hold for V1 — no item columns are in match_players staging yet, so nothing joins to it. deterministic hash of _dlt_id, stable across view re-runs</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>not_null, unique</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
@@ -3200,10 +3204,14 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Matches item_0-item_5 etc. on match players (not yet in staging scope)</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr"/>
+          <t>the item's real numeric id (1 to 4302 in our data). it's what item_0–item_5 on match players would point at if we ever bring those in — nothing to relationship-test against yet</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>not_null, unique — 501 of 501 populated and all distinct</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" s="6" t="inlineStr">
@@ -3248,15 +3256,19 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Rename dname -&gt; item_name</t>
+          <t>Rename dname -&gt; item_name, TRIM only — don't capitalize</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>10 of 501 items have no display name in current data</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr"/>
+          <t>10 of 501 items have no display name — that's the source (things like greater_mango, horizon, recipe_wraith_pact), not a bug, so it stays nullable. names also repeat across upgrade levels (Dagon shows up 5 times, Necronomicon 3), so it isn't a unique key either. leaving the casing alone, same reasoning as hero_name</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>no not_null (10 real nulls) and no unique (Dagon x5) — use dbt_utils.not_null_proportion(at_least=0.9) instead: tolerates the real nulls but still catches the column going empty (98% populated today)</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
@@ -3306,10 +3318,14 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>10 of 501 items have no cost in current data</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr"/>
+          <t>10 of 501 have no cost, and 197 cost exactly 0 (175 of those have no quality tag) — 0 is a real value here, don't treat it as missing. the missing-cost items are mostly different ones from the missing-name items, only 2 are missing both</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0) — non-negative, not 'positive', since 197 items really do cost 0. no upper cap on purpose: 154 of 491 items are already over 1000 (Dagon is 7650) and prices shift every patch, so a fixed ceiling would just break on legit changes. no not_null since the 10 nulls are real — dbt_utils.not_null_proportion(at_least=0.9) instead so a wholesale collapse still gets caught</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
@@ -3357,8 +3373,12 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
-      <c r="K6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>not_null, unique</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
@@ -3406,8 +3426,12 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>not_null</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K7"/>

</xml_diff>

<commit_message>
docs:update sttm source to staging
</commit_message>
<xml_diff>
--- a/docs/sttm_raw_to_staging.xlsx
+++ b/docs/sttm_raw_to_staging.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="-28920" yWindow="8130" windowWidth="29040" windowHeight="15720" tabRatio="600" firstSheet="0" activeTab="8" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet name="README" sheetId="1" state="visible" r:id="rId1"/>
@@ -29,7 +28,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'match_players'!$A$1:$K$29</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="9" hidden="1">'match_gold_advantage'!$A$1:$K$6</definedName>
   </definedNames>
-  <calcPr calcId="124519" fullCalcOnLoad="1"/>
+  <calcPr calcId="0" fullCalcOnLoad="1"/>
 </workbook>
 </file>
 
@@ -45,18 +44,22 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00FFFFFF"/>
+      <color rgb="FFFFFFFF"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="13"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <sz val="11"/>
     </font>
     <font>
+      <name val="Calibri"/>
       <b val="1"/>
       <sz val="11"/>
     </font>
@@ -70,22 +73,22 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="001F2937"/>
+        <fgColor rgb="FF1F2937"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFF3CD"/>
+        <fgColor rgb="FFFFF3CD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00E7F0FA"/>
+        <fgColor rgb="FFE7F0FA"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FCE4D6"/>
+        <fgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
   </fills>
@@ -99,17 +102,18 @@
     </border>
     <border>
       <left style="thin">
-        <color rgb="00D0D0D0"/>
+        <color rgb="FFD0D0D0"/>
       </left>
       <right style="thin">
-        <color rgb="00D0D0D0"/>
+        <color rgb="FFD0D0D0"/>
       </right>
       <top style="thin">
-        <color rgb="00D0D0D0"/>
+        <color rgb="FFD0D0D0"/>
       </top>
       <bottom style="thin">
-        <color rgb="00D0D0D0"/>
+        <color rgb="FFD0D0D0"/>
       </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -143,7 +147,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -506,13 +510,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A17"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <dimension ref="A1:A23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
     <col width="110" customWidth="1" min="1" max="1"/>
   </cols>
   <sheetData>
-    <row r="1">
+    <row r="1" ht="17" customHeight="1">
       <c r="A1" s="1" t="inlineStr">
         <is>
           <t>Source-to-Target Mapping — Raw to Staging</t>
@@ -520,7 +524,7 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="inlineStr"/>
+      <c r="A2" s="2" t="n"/>
     </row>
     <row r="3">
       <c r="A3" s="2" t="inlineStr">
@@ -530,7 +534,7 @@
       </c>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="inlineStr"/>
+      <c r="A4" s="2" t="n"/>
     </row>
     <row r="5">
       <c r="A5" s="3" t="inlineStr">
@@ -561,7 +565,7 @@
       </c>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="inlineStr"/>
+      <c r="A9" s="2" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
@@ -570,7 +574,7 @@
         </is>
       </c>
     </row>
-    <row r="11">
+    <row r="11" ht="29" customHeight="1">
       <c r="A11" s="2" t="inlineStr">
         <is>
           <t xml:space="preserve">  staging_&lt;table&gt;_id = generate_surrogate_key(['_dlt_id']) — our own row key, not dlt_id itself, unique even when the business key repeats (matches does this)</t>
@@ -592,9 +596,9 @@
       </c>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="inlineStr"/>
-    </row>
-    <row r="15">
+      <c r="A14" s="2" t="n"/>
+    </row>
+    <row r="15" ht="29" customHeight="1">
       <c r="A15" s="2" t="inlineStr">
         <is>
           <t>The Nullable columns are from actually querying Snowflake, not guessing off the declared schema — Snowflake/dlt don't enforce NOT NULL on inferred columns, so the schema alone would tell you almost nothing is required.</t>
@@ -602,12 +606,47 @@
       </c>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="inlineStr"/>
+      <c r="A16" s="2" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
           <t>Companion docs: docs/bus_matrix.md, docs/ingestion_architecture.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>Business-rule tests beyond the routine per-field checks — 3 generic, 1 true singular:</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  1. (generic) matches.start_time not in the future — dbt_utils.expression_is_true, source yml</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  2. (generic) matches__players.rank_tier — two separate table-level dbt_utils.expression_is_true tests in the source yml: floor(rank_tier / 10) between 1 and 8 (bracket digit), and mod(rank_tier, 10) between 0 and 5 (star digit). Kept as two so a failure tells you which digit is wrong. Table-level because column-level expression_is_true only appends text after the column name — it can't wrap floor()/mod() around it.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  3. (generic) matches__players player_slot is unique per match — dbt_utils.unique_combination_of_columns on (_dlt_parent_id, player_slot), source yml. One player per slot per match, not one slot per player overall.</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="2" t="inlineStr">
+        <is>
+          <t xml:space="preserve">  4. (singular) matches__players has exactly 10 rows per match (5v5) — the only one of these that's a real singular test: tests/singular/assert_ten_players_per_match.sql. dbt has no ready-made generic test for 'row count per group', which is why this one needed its own SQL file instead of a macro.</t>
         </is>
       </c>
     </row>
@@ -623,10 +662,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -695,10 +733,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.5" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__match_gold_advantage</t>
+          <t>stg_matches__match_gold_advantage</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -752,10 +790,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="101.5" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>stg_opendota__match_gold_advantage</t>
+          <t>stg_matches__match_gold_advantage</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -775,190 +813,190 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
+          <t>matches (parent, joined on _dlt_parent_id)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>match_id</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>LEFT JOIN to stg_matches__matches on _dlt_parent_id = matches.dlt_row_id, return matches.source_match_id</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>same reasoning as hero_roles — has to be a LEFT JOIN or an orphaned gold-advantage row would just silently vanish instead of showing up as a real problem</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>not_null, relationships: raw _dlt_parent_id -&gt; matches._dlt_id (this check lives in the source yml). It points at the parent row's dlt id, not match_id, because match_id repeats in the append-only matches table so it can't identify one parent row. After the LEFT JOIN, not_null on source_match_id catches any orphan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="101.5" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_gold_advantage</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>minute_mark</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
           <t>matches__radiant_gold_adv</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>_dlt_parent_id</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>_dlt_list_idx</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Rename</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>this is the actual minute of the match — the whole point of staging this table, don't drop it</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0) — can't be negative, it's an array position, plus a custom test checking minute_mark &lt;= matches.duration/60 for that match — checked all 83 current rows against their real match duration and none violate it, so this is a real invariant, not just a made-up ceiling</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="29" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_gold_advantage</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>radiant_gold_advantage</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>matches__radiant_gold_adv</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>Rename</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>negative means Dire's actually ahead</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>not_null</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="29" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_gold_advantage</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>dlt_row_id</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
+        <is>
+          <t>matches__radiant_gold_adv</t>
+        </is>
+      </c>
+      <c r="F6" s="6" t="inlineStr">
+        <is>
+          <t>_dlt_id</t>
+        </is>
+      </c>
+      <c r="G6" s="6" t="inlineStr">
         <is>
           <t>TEXT</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>LEFT JOIN to stg_opendota__matches on _dlt_parent_id = matches.dlt_row_id, return matches.source_match_id</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>same reasoning as hero_roles — has to be a LEFT JOIN or an orphaned gold-advantage row would just silently vanish instead of showing up as a real problem</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>not_null, relationships -&gt; stg_opendota__matches.source_match_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_gold_advantage</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>minute_mark</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
-        <is>
-          <t>matches__radiant_gold_adv</t>
-        </is>
-      </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>_dlt_list_idx</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Rename</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>this is the actual minute of the match — the whole point of staging this table, don't drop it</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>not_null, accepted_range(min_value=0) — can't be negative, it's an array position, plus a custom test checking minute_mark &lt;= matches.duration/60 for that match — checked all 83 current rows against their real match duration and none violate it, so this is a real invariant, not just a made-up ceiling</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_gold_advantage</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>radiant_gold_advantage</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>matches__radiant_gold_adv</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Rename</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>negative means Dire's actually ahead</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
-        <is>
-          <t>not_null</t>
-        </is>
-      </c>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_gold_advantage</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>dlt_row_id</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
-        <is>
-          <t>matches__radiant_gold_adv</t>
-        </is>
-      </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>_dlt_id</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
       <c r="H6" s="6" t="inlineStr">
         <is>
           <t>NO</t>
@@ -969,7 +1007,7 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
@@ -989,10 +1027,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K9"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -1061,10 +1098,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1121,7 +1158,7 @@
     <row r="3">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -1175,10 +1212,10 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="43.5" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -1232,10 +1269,10 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="29" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -1292,7 +1329,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -1346,10 +1383,10 @@
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -1406,7 +1443,7 @@
     <row r="8">
       <c r="A8" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B8" s="6" t="inlineStr">
@@ -1449,17 +1486,17 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr"/>
+      <c r="J8" s="6" t="n"/>
       <c r="K8" s="6" t="inlineStr">
         <is>
           <t>not_null</t>
         </is>
       </c>
     </row>
-    <row r="9">
+    <row r="9" ht="29" customHeight="1">
       <c r="A9" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__heroes</t>
+          <t>stg_master_data__heroes</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
@@ -1526,10 +1563,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K5"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -1598,10 +1634,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.5" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__hero_roles</t>
+          <t>stg_master_data__heroes_roles</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1655,10 +1691,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="101.5" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>stg_opendota__hero_roles</t>
+          <t>stg_master_data__heroes_roles</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -1678,133 +1714,133 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
+          <t>heroes (parent, joined on _dlt_parent_id)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>id</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>LEFT JOIN to stg_master_data__heroes on _dlt_parent_id = heroes.dlt_row_id, return heroes.source_hero_id</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>has to be a LEFT JOIN — an INNER JOIN would just quietly drop any role that can't find its hero, and we'd never notice. that breaks the whole raw-immutability thing</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>not_null, relationships: raw _dlt_parent_id -&gt; heroes._dlt_id (this check lives in the source yml). It points at the parent row's dlt id because that's what _dlt_parent_id actually references, the hero id is a separate business key. After the LEFT JOIN, not_null on source_hero_id catches any orphan</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="43.5" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>stg_master_data__heroes_roles</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>role_name</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>STRING</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
           <t>heroes__roles</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>_dlt_parent_id</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
+        <is>
+          <t>value</t>
+        </is>
+      </c>
+      <c r="G4" s="6" t="inlineStr">
         <is>
           <t>TEXT</t>
         </is>
       </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>LEFT JOIN to stg_opendota__heroes on _dlt_parent_id = heroes.dlt_row_id, return heroes.source_hero_id</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>has to be a LEFT JOIN — an INNER JOIN would just quietly drop any role that can't find its hero, and we'd never notice. that breaks the whole raw-immutability thing</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr">
-        <is>
-          <t>not_null, relationships -&gt; stg_opendota__heroes.source_hero_id (really just checking the LEFT JOIN actually found a match)</t>
-        </is>
-      </c>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__hero_roles</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
-        <is>
-          <t>role_name</t>
-        </is>
-      </c>
-      <c r="C4" s="6" t="inlineStr">
+      <c r="H4" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Rename value -&gt; role_name, TRIM only — don't capitalize</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>e.g. Carry, Support, Nuker — already cased fine as it comes in</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_values: ['Carry', 'Disabler', 'Durable', 'Escape', 'Initiator', 'Nuker', 'Pusher', 'Support']</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="29" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>stg_master_data__heroes_roles</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>dlt_row_id</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
         <is>
           <t>STRING</t>
         </is>
       </c>
-      <c r="D4" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>heroes__roles</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>value</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>_dlt_id</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
         <is>
           <t>TEXT</t>
         </is>
       </c>
-      <c r="H4" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Rename value -&gt; role_name, TRIM only — don't capitalize</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>e.g. Carry, Support, Nuker — already cased fine as it comes in</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr">
-        <is>
-          <t>not_null, accepted_values: ['Carry', 'Disabler', 'Durable', 'Escape', 'Initiator', 'Nuker', 'Pusher', 'Support']</t>
-        </is>
-      </c>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__hero_roles</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>dlt_row_id</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
-        <is>
-          <t>heroes__roles</t>
-        </is>
-      </c>
-      <c r="F5" s="6" t="inlineStr">
-        <is>
-          <t>_dlt_id</t>
-        </is>
-      </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
       <c r="H5" s="6" t="inlineStr">
         <is>
           <t>NO</t>
@@ -1815,7 +1851,7 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
@@ -1835,10 +1871,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -1907,10 +1942,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.5" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__game_modes</t>
+          <t>stg_master_data__game_mode</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -1964,10 +1999,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="29" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__game_modes</t>
+          <t>stg_master_data__game_mode</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -2010,17 +2045,17 @@
           <t>Rename id -&gt; source_game_mode_id</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="72.5" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__game_modes</t>
+          <t>stg_master_data__game_mode</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -2074,10 +2109,10 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="43.5" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__game_modes</t>
+          <t>stg_master_data__game_mode</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2131,10 +2166,10 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__game_modes</t>
+          <t>stg_master_data__game_mode</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -2177,17 +2212,17 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__game_modes</t>
+          <t>stg_master_data__game_mode</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2230,7 +2265,7 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="inlineStr">
         <is>
           <t>not_null</t>
@@ -2250,10 +2285,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -2322,10 +2356,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.5" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__lobby_types</t>
+          <t>stg_master_data__lobby_type</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -2379,10 +2413,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="29" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__lobby_types</t>
+          <t>stg_master_data__lobby_type</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -2425,17 +2459,17 @@
           <t>Rename id -&gt; source_lobby_type_id</t>
         </is>
       </c>
-      <c r="J3" s="6" t="inlineStr"/>
+      <c r="J3" s="6" t="n"/>
       <c r="K3" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="72.5" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__lobby_types</t>
+          <t>stg_master_data__lobby_type</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -2489,10 +2523,10 @@
         </is>
       </c>
     </row>
-    <row r="5">
+    <row r="5" ht="43.5" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__lobby_types</t>
+          <t>stg_master_data__lobby_type</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2546,10 +2580,10 @@
         </is>
       </c>
     </row>
-    <row r="6">
+    <row r="6" ht="29" customHeight="1">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__lobby_types</t>
+          <t>stg_master_data__lobby_type</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -2592,17 +2626,17 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
         </is>
       </c>
     </row>
-    <row r="7">
+    <row r="7" ht="29" customHeight="1">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__lobby_types</t>
+          <t>stg_master_data__lobby_type</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -2645,7 +2679,7 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n"/>
       <c r="K7" s="6" t="inlineStr">
         <is>
           <t>not_null</t>
@@ -2665,10 +2699,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K6"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -2737,10 +2770,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="43.5" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__regions</t>
+          <t>stg_master_data__region</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -2794,10 +2827,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="43.5" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__regions</t>
+          <t>stg_master_data__region</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -2851,10 +2884,10 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="58" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__regions</t>
+          <t>stg_master_data__region</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -2911,7 +2944,7 @@
     <row r="5">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__regions</t>
+          <t>stg_master_data__region</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -2954,7 +2987,7 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J5" s="6" t="inlineStr"/>
+      <c r="J5" s="6" t="n"/>
       <c r="K5" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
@@ -2964,7 +2997,7 @@
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__regions</t>
+          <t>stg_master_data__region</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -3007,7 +3040,7 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="n"/>
       <c r="K6" s="6" t="inlineStr">
         <is>
           <t>not_null</t>
@@ -3027,10 +3060,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K7"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -3099,10 +3131,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="72.5" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__items</t>
+          <t>stg_master_data__items</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -3147,15 +3179,19 @@
       </c>
       <c r="J2" s="5" t="inlineStr">
         <is>
-          <t>New technical key, not dlt_id itself</t>
-        </is>
-      </c>
-      <c r="K2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3">
+          <t>would carry through as dim_item's key at mart, but dim_item is on hold for V1 — no item columns are in match_players staging yet, so nothing joins to it. deterministic hash of _dlt_id, stable across view re-runs</t>
+        </is>
+      </c>
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>not_null, unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="58" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__items</t>
+          <t>stg_master_data__items</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -3200,15 +3236,19 @@
       </c>
       <c r="J3" s="6" t="inlineStr">
         <is>
-          <t>Matches item_0-item_5 etc. on match players (not yet in staging scope)</t>
-        </is>
-      </c>
-      <c r="K3" s="6" t="inlineStr"/>
-    </row>
-    <row r="4">
+          <t>the item's real numeric id (1 to 4302 in our data). it's what item_0–item_5 on match players would point at if we ever bring those in — nothing to relationship-test against yet</t>
+        </is>
+      </c>
+      <c r="K3" s="6" t="inlineStr">
+        <is>
+          <t>not_null, unique — 501 of 501 populated and all distinct</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="101.5" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__items</t>
+          <t>stg_master_data__items</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -3248,20 +3288,24 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Rename dname -&gt; item_name</t>
+          <t>Rename dname -&gt; item_name, TRIM only — don't capitalize</t>
         </is>
       </c>
       <c r="J4" s="6" t="inlineStr">
         <is>
-          <t>10 of 501 items have no display name in current data</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5">
+          <t>10 of 501 items have no display name — that's the source (things like greater_mango, horizon, recipe_wraith_pact), not a bug, so it stays nullable. names also repeat across upgrade levels (Dagon shows up 5 times, Necronomicon 3), so it isn't a unique key either. leaving the casing alone, same reasoning as hero_name</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>no not_null (10 real nulls) and no unique (Dagon x5) — use dbt_utils.not_null_proportion(at_least=0.9) instead: tolerates the real nulls but still catches the column going empty (98% populated today)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="145" customHeight="1">
       <c r="A5" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__items</t>
+          <t>stg_master_data__items</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
@@ -3306,15 +3350,19 @@
       </c>
       <c r="J5" s="6" t="inlineStr">
         <is>
-          <t>10 of 501 items have no cost in current data</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr"/>
+          <t>10 of 501 have no cost, and 197 cost exactly 0 (175 of those have no quality tag) — 0 is a real value here, don't treat it as missing. the missing-cost items are mostly different ones from the missing-name items, only 2 are missing both</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0) — non-negative, not 'positive', since 197 items really do cost 0. no upper cap on purpose: 154 of 491 items are already over 1000 (Dagon is 7650) and prices shift every patch, so a fixed ceiling would just break on legit changes. no not_null since the 10 nulls are real — dbt_utils.not_null_proportion(at_least=0.9) instead so a wholesale collapse still gets caught</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__items</t>
+          <t>stg_master_data__items</t>
         </is>
       </c>
       <c r="B6" s="6" t="inlineStr">
@@ -3357,13 +3405,17 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J6" s="6" t="inlineStr"/>
-      <c r="K6" s="6" t="inlineStr"/>
+      <c r="J6" s="6" t="n"/>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>not_null, unique</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__items</t>
+          <t>stg_master_data__items</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
@@ -3406,8 +3458,12 @@
           <t>Rename, lineage only</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
+      <c r="J7" s="6" t="n"/>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>not_null</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K7"/>
@@ -3422,10 +3478,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K23"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -3494,10 +3549,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="58" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -3551,10 +3606,10 @@
         </is>
       </c>
     </row>
-    <row r="3">
+    <row r="3" ht="43.5" customHeight="1">
       <c r="A3" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B3" s="6" t="inlineStr">
@@ -3594,7 +3649,7 @@
       </c>
       <c r="I3" s="6" t="inlineStr">
         <is>
-          <t>Rename match_id -&gt; source_match_id; CAST to NUMBER(38,0)</t>
+          <t>Rename match_id -&gt; source_match_id</t>
         </is>
       </c>
       <c r="J3" s="6" t="inlineStr">
@@ -3608,10 +3663,10 @@
         </is>
       </c>
     </row>
-    <row r="4">
+    <row r="4" ht="29" customHeight="1">
       <c r="A4" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B4" s="6" t="inlineStr">
@@ -3651,446 +3706,450 @@
       </c>
       <c r="I4" s="6" t="inlineStr">
         <is>
-          <t>Convert Unix timestamp; derive match_date</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr"/>
+          <t>to_timestamp(start_time) — Unix seconds, so the result is UTC</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>the calendar date lives in match_date, right below, derived from the same timestamp</t>
+        </is>
+      </c>
       <c r="K4" s="6" t="inlineStr">
         <is>
+          <t>not_null — also checked not in the future: start_time &lt;= current_timestamp (generic test, dbt_utils.expression_is_true, source yml)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="29" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>match_date</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>DATE</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>matches</t>
+        </is>
+      </c>
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>start_time</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>to_date(to_timestamp(start_time)) — the UTC calendar date of the start</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>feeds match_date_key -&gt; dim_date at mart</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
           <t>not_null</t>
         </is>
       </c>
     </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>duration_seconds</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E5" s="6" t="inlineStr">
+    <row r="6" ht="72.5" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>duration_min</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER(26,0)</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>duration</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>Rename; derive duration_minutes</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>confirmed this is genuinely in seconds (longest match in our data is 1182 sec ~ 19.7 min, not 1182 min) — don't accidentally treat it as minutes downstream</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>round(duration / 60, 0) — seconds to whole minutes</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>raw duration is in seconds (longest match in our data was 1182 sec, about 19.7 min, not 1182 min), so the /60 is what makes it minutes. rounded to whole minutes on purpose, no decimals — the exact seconds stay in raw if we ever want them back</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0)</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>winning_team</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>STRING</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
+    <row r="7" ht="43.5" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>radiant_win</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>radiant_win</t>
         </is>
       </c>
-      <c r="G6" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>Cast boolean; derive 'radiant'/'dire' lowercase</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>lowercase on purpose so it lines up exactly with dim_team's keys at mart — no case mismatch on the join</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr">
-        <is>
-          <t>not_null, accepted_values: ['radiant', 'dire']</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Keep as boolean, no derived label in staging</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>stays a real true/false boolean here. the radiant/dire winner label that lines up with dim_team gets derived at mart (winner_team_key), not in staging</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>not_null — no accepted_values, it's a real BOOLEAN so it can only be true or false</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="29" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
         <is>
           <t>radiant_tower_status_bitmask</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
         <is>
           <t>tower_status_radiant</t>
         </is>
       </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
         <is>
           <t>Rename, keep as raw integer for now</t>
         </is>
       </c>
-      <c r="J7" s="6" t="inlineStr">
+      <c r="J8" s="6" t="inlineStr">
         <is>
           <t>decode into a tower count at mart if needed — leaving it as the raw bitmask in staging</t>
         </is>
       </c>
-      <c r="K7" s="6" t="inlineStr">
+      <c r="K8" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0, max_value=2047) — 11 towers</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
+    <row r="9" ht="29" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
         <is>
           <t>dire_tower_status_bitmask</t>
         </is>
       </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>tower_status_dire</t>
         </is>
       </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>Rename, keep as raw integer for now</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>same as radiant — decode at mart, not here</t>
         </is>
       </c>
-      <c r="K8" s="6" t="inlineStr">
+      <c r="K9" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0, max_value=2047) — 11 towers</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+    <row r="10" ht="43.5" customHeight="1">
+      <c r="A10" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B10" s="6" t="inlineStr">
         <is>
           <t>radiant_barracks_status_bitmask</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
+      <c r="C10" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D10" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E10" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F9" s="6" t="inlineStr">
+      <c r="F10" s="6" t="inlineStr">
         <is>
           <t>barracks_status_radiant</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H9" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I9" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H10" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I10" s="6" t="inlineStr">
         <is>
           <t>Rename, keep as raw integer for now</t>
         </is>
       </c>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>6 barracks per side (2 per lane x 3 lanes), so this maxes out at 63, not 2047 like the towers do — different bitmask, don't mix up the ranges</t>
         </is>
       </c>
-      <c r="K9" s="6" t="inlineStr">
+      <c r="K10" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0, max_value=63) — 6 barracks, NOT 2047, don't reuse the tower range here</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B10" s="6" t="inlineStr">
+    <row r="11" ht="29" customHeight="1">
+      <c r="A11" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>dire_barracks_status_bitmask</t>
         </is>
       </c>
-      <c r="C10" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D10" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E10" s="6" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F10" s="6" t="inlineStr">
+      <c r="F11" s="6" t="inlineStr">
         <is>
           <t>barracks_status_dire</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H10" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H11" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Rename, keep as raw integer for now</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>same as radiant barracks — maxes out at 63</t>
         </is>
       </c>
-      <c r="K10" s="6" t="inlineStr">
+      <c r="K11" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0, max_value=63) — 6 barracks</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B11" s="6" t="inlineStr">
-        <is>
-          <t>first_blood_time_seconds</t>
-        </is>
-      </c>
-      <c r="C11" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D11" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E11" s="6" t="inlineStr">
+    <row r="12" ht="72.5" customHeight="1">
+      <c r="A12" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B12" s="6" t="inlineStr">
+        <is>
+          <t>first_blood_time_sec</t>
+        </is>
+      </c>
+      <c r="C12" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D12" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E12" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F11" s="6" t="inlineStr">
+      <c r="F12" s="6" t="inlineStr">
         <is>
           <t>first_blood_time</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H11" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I11" s="6" t="inlineStr">
-        <is>
-          <t>Rename, keep in seconds — don't round to minutes</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr">
-        <is>
-          <t>checked: 74 of 151 matches have first blood under 60 seconds, so rounding to whole minutes would flatten half the data to zero. dashboard KPI: Avg First Blood Time</t>
-        </is>
-      </c>
-      <c r="K11" s="6" t="inlineStr">
-        <is>
-          <t>not_null, accepted_range(min_value=0)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B12" s="6" t="inlineStr">
-        <is>
-          <t>radiant_kill_count</t>
-        </is>
-      </c>
-      <c r="C12" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D12" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E12" s="6" t="inlineStr">
-        <is>
-          <t>matches</t>
-        </is>
-      </c>
-      <c r="F12" s="6" t="inlineStr">
-        <is>
-          <t>radiant_score</t>
-        </is>
-      </c>
       <c r="G12" s="6" t="inlineStr">
         <is>
           <t>NUMBER</t>
@@ -4103,10 +4162,14 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Rename</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr"/>
+          <t>Rename only — stays in seconds</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="inlineStr">
+        <is>
+          <t>kept in seconds on purpose: about half the matches (74 of 151 when checked) had first blood under a minute, so in minutes they'd all be tiny fractions. convert at mart if the dashboard wants minutes. dashboard KPI: Avg First Blood Time</t>
+        </is>
+      </c>
       <c r="K12" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0)</t>
@@ -4116,12 +4179,12 @@
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
         <is>
-          <t>dire_kill_count</t>
+          <t>radiant_kill_count</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
@@ -4141,7 +4204,7 @@
       </c>
       <c r="F13" s="6" t="inlineStr">
         <is>
-          <t>dire_score</t>
+          <t>radiant_score</t>
         </is>
       </c>
       <c r="G13" s="6" t="inlineStr">
@@ -4159,7 +4222,7 @@
           <t>Rename</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="n"/>
       <c r="K13" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0)</t>
@@ -4169,463 +4232,459 @@
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
+          <t>dire_kill_count</t>
+        </is>
+      </c>
+      <c r="C14" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D14" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E14" s="6" t="inlineStr">
+        <is>
+          <t>matches</t>
+        </is>
+      </c>
+      <c r="F14" s="6" t="inlineStr">
+        <is>
+          <t>dire_score</t>
+        </is>
+      </c>
+      <c r="G14" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I14" s="6" t="inlineStr">
+        <is>
+          <t>Rename</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="29" customHeight="1">
+      <c r="A15" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
           <t>human_players</t>
         </is>
       </c>
-      <c r="C14" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D14" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E14" s="6" t="inlineStr">
+      <c r="C15" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D15" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E15" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F14" s="6" t="inlineStr">
+      <c r="F15" s="6" t="inlineStr">
         <is>
           <t>human_players</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H14" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I14" s="6" t="inlineStr">
-        <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H15" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I15" s="6" t="inlineStr">
+        <is>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>not shown on the dashboard, but this is how we'd flag broken/incomplete matches later</t>
         </is>
       </c>
-      <c r="K14" s="6" t="inlineStr">
+      <c r="K15" s="6" t="inlineStr">
         <is>
           <t>not_null, accepted_range(min_value=0, max_value=10)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B15" s="6" t="inlineStr">
+    <row r="16" ht="72.5" customHeight="1">
+      <c r="A16" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B16" s="6" t="inlineStr">
         <is>
           <t>source_lobby_type_id</t>
         </is>
       </c>
-      <c r="C15" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D15" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E15" s="6" t="inlineStr">
+      <c r="C16" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D16" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E16" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F15" s="6" t="inlineStr">
+      <c r="F16" s="6" t="inlineStr">
         <is>
           <t>lobby_type</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H15" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I15" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H16" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I16" s="6" t="inlineStr">
         <is>
           <t>Rename only — this is already the literal id, no lookup needed here</t>
         </is>
       </c>
-      <c r="J15" s="6" t="inlineStr">
-        <is>
-          <t>joins to stg_opendota__lobby_types.source_lobby_type_id</t>
-        </is>
-      </c>
-      <c r="K15" s="6" t="inlineStr">
-        <is>
-          <t>not_null, relationships -&gt; stg_opendota__lobby_types.source_lobby_type_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B16" s="6" t="inlineStr">
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>joins to stg_master_data__lobby_type.source_lobby_type_id</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>not_null, relationships: raw matches.lobby_type -&gt; constants_lobby_type.id — checked against the raw lookup in the source yml, not against staging (0 orphans today)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="72.5" customHeight="1">
+      <c r="A17" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
         <is>
           <t>source_game_mode_id</t>
         </is>
       </c>
-      <c r="C16" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D16" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E16" s="6" t="inlineStr">
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F16" s="6" t="inlineStr">
+      <c r="F17" s="6" t="inlineStr">
         <is>
           <t>game_mode</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H16" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H17" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Rename only — this is already the literal id, no lookup needed here</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
-        <is>
-          <t>joins to stg_opendota__game_modes.source_game_mode_id</t>
-        </is>
-      </c>
-      <c r="K16" s="6" t="inlineStr">
-        <is>
-          <t>not_null, relationships -&gt; stg_opendota__game_modes.source_game_mode_id</t>
-        </is>
-      </c>
-    </row>
-    <row r="17">
-      <c r="A17" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B17" s="6" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
+        <is>
+          <t>joins to stg_master_data__game_mode.source_game_mode_id</t>
+        </is>
+      </c>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>not_null, relationships: raw matches.game_mode -&gt; constants_game_mode.id — checked against the raw lookup in the source yml, not against staging (0 orphans today)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="116" customHeight="1">
+      <c r="A18" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B18" s="6" t="inlineStr">
         <is>
           <t>source_region_id</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="C18" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D18" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F17" s="6" t="inlineStr">
+      <c r="F18" s="6" t="inlineStr">
         <is>
           <t>region</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
-        <is>
-          <t>Rename; joins to stg_opendota__regions.source_region_id</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr">
-        <is>
-          <t>genuinely nullable — 117 of 151 matches have it populated, not every response includes a region</t>
-        </is>
-      </c>
-      <c r="K17" s="6" t="inlineStr">
-        <is>
-          <t>relationships -&gt; stg_opendota__regions.source_region_id (no not_null, it's genuinely optional)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18">
-      <c r="A18" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B18" s="6" t="inlineStr">
-        <is>
-          <t>patch_id</t>
-        </is>
-      </c>
-      <c r="C18" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D18" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E18" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
+        <is>
+          <t>Rename; joins to stg_master_data__region.source_region_id</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="inlineStr">
+        <is>
+          <t>genuinely nullable — 137 of 174 matches have it populated (37 don't), not every response includes a region</t>
+        </is>
+      </c>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>relationships: raw matches.region -&gt; constants_region.id — checked against the raw lookup in the source yml, not against staging (0 orphans today). no not_null, region is genuinely optional. raw constants_region.id is TEXT while matches.region is NUMBER, Snowflake casts it implicitly so it works, just know it's there</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="29" customHeight="1">
+      <c r="A19" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B19" s="6" t="inlineStr">
+        <is>
+          <t>patch</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
         <is>
           <t>matches</t>
         </is>
       </c>
-      <c r="F18" s="6" t="inlineStr">
+      <c r="F19" s="6" t="inlineStr">
         <is>
           <t>patch</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H18" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I18" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H19" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I19" s="6" t="inlineStr">
+        <is>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="inlineStr">
+        <is>
+          <t>dashboard filter: Patch. no _id suffix on purpose — there's no patch table for it to point at</t>
+        </is>
+      </c>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>not_null</t>
+        </is>
+      </c>
+    </row>
+    <row r="20" ht="58" customHeight="1">
+      <c r="A20" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B20" s="6" t="inlineStr">
+        <is>
+          <t>parse_version</t>
+        </is>
+      </c>
+      <c r="C20" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D20" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E20" s="6" t="inlineStr">
+        <is>
+          <t>matches</t>
+        </is>
+      </c>
+      <c r="F20" s="6" t="inlineStr">
+        <is>
+          <t>version</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr">
         <is>
           <t>Rename</t>
         </is>
       </c>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>dashboard filter: Patch</t>
-        </is>
-      </c>
-      <c r="K18" s="6" t="inlineStr">
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>only 5 of 151 matches have this populated — most of what we've pulled isn't fully parsed yet. needed for the int_matches__latest_complete dedup logic, alongside is_parsed</t>
+        </is>
+      </c>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>no not_null — mostly empty right now since most matches aren't parsed yet, that's expected</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="29" customHeight="1">
+      <c r="A21" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__matches</t>
+        </is>
+      </c>
+      <c r="B21" s="6" t="inlineStr">
+        <is>
+          <t>is_parsed</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>matches</t>
+        </is>
+      </c>
+      <c r="F21" s="6" t="inlineStr">
+        <is>
+          <t>od_data__has_parsed</t>
+        </is>
+      </c>
+      <c r="G21" s="6" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="H21" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I21" s="6" t="inlineStr">
+        <is>
+          <t>Rename only</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="inlineStr">
+        <is>
+          <t>the important one — this is what picks the preferred version of a match</t>
+        </is>
+      </c>
+      <c r="K21" s="6" t="inlineStr">
         <is>
           <t>not_null</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="A19" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B19" s="6" t="inlineStr">
-        <is>
-          <t>parse_version</t>
-        </is>
-      </c>
-      <c r="C19" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D19" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr">
-        <is>
-          <t>matches</t>
-        </is>
-      </c>
-      <c r="F19" s="6" t="inlineStr">
-        <is>
-          <t>version</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I19" s="6" t="inlineStr">
-        <is>
-          <t>Rename</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr">
-        <is>
-          <t>only 5 of 151 matches have this populated — most of what we've pulled isn't fully parsed yet. needed for the int_matches__latest_complete dedup logic, alongside is_parsed</t>
-        </is>
-      </c>
-      <c r="K19" s="6" t="inlineStr">
-        <is>
-          <t>no not_null — mostly empty right now since most matches aren't parsed yet, that's expected</t>
-        </is>
-      </c>
-    </row>
-    <row r="20">
-      <c r="A20" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B20" s="6" t="inlineStr">
-        <is>
-          <t>has_game_coordinator_data</t>
-        </is>
-      </c>
-      <c r="C20" s="6" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="D20" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E20" s="6" t="inlineStr">
-        <is>
-          <t>matches</t>
-        </is>
-      </c>
-      <c r="F20" s="6" t="inlineStr">
-        <is>
-          <t>od_data__has_gcdata</t>
-        </is>
-      </c>
-      <c r="G20" s="6" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="H20" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I20" s="6" t="inlineStr">
-        <is>
-          <t>Rename, cast boolean</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr">
-        <is>
-          <t>actually varies in our data (16 true, 135 false), unlike has_api/has_archive which we dropped for being constant — this one's worth keeping</t>
-        </is>
-      </c>
-      <c r="K20" s="6" t="inlineStr">
-        <is>
-          <t>not_null</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__matches</t>
-        </is>
-      </c>
-      <c r="B21" s="6" t="inlineStr">
-        <is>
-          <t>is_parsed</t>
-        </is>
-      </c>
-      <c r="C21" s="6" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="D21" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E21" s="6" t="inlineStr">
-        <is>
-          <t>matches</t>
-        </is>
-      </c>
-      <c r="F21" s="6" t="inlineStr">
-        <is>
-          <t>od_data__has_parsed</t>
-        </is>
-      </c>
-      <c r="G21" s="6" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
-      <c r="H21" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I21" s="6" t="inlineStr">
-        <is>
-          <t>Rename, cast boolean</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr">
-        <is>
-          <t>the important one — this is what picks the preferred version of a match</t>
-        </is>
-      </c>
-      <c r="K21" s="6" t="inlineStr">
-        <is>
-          <t>not_null</t>
-        </is>
-      </c>
-    </row>
-    <row r="22">
+    <row r="22" ht="29" customHeight="1">
       <c r="A22" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B22" s="6" t="inlineStr">
@@ -4682,7 +4741,7 @@
     <row r="23">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__matches</t>
+          <t>stg_matches__matches</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -4749,10 +4808,9 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:K29"/>
-  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="14.5"/>
   <cols>
-    <col width="26" customWidth="1" min="1" max="1"/>
-    <col width="26" customWidth="1" min="2" max="2"/>
+    <col width="26" customWidth="1" min="1" max="2"/>
     <col width="16" customWidth="1" min="3" max="3"/>
     <col width="12" customWidth="1" min="4" max="4"/>
     <col width="22" customWidth="1" min="5" max="5"/>
@@ -4821,10 +4879,10 @@
         </is>
       </c>
     </row>
-    <row r="2">
+    <row r="2" ht="29" customHeight="1">
       <c r="A2" s="5" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B2" s="5" t="inlineStr">
@@ -4872,12 +4930,16 @@
           <t>carries through as fact_match_players' key at mart — deterministic hash of _dlt_id</t>
         </is>
       </c>
-      <c r="K2" s="5" t="inlineStr"/>
-    </row>
-    <row r="3">
+      <c r="K2" s="5" t="inlineStr">
+        <is>
+          <t>not_null, unique</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="101.5" customHeight="1">
       <c r="A3" s="7" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B3" s="7" t="inlineStr">
@@ -4897,329 +4959,361 @@
       </c>
       <c r="E3" s="7" t="inlineStr">
         <is>
+          <t>matches (parent, joined on _dlt_parent_id)</t>
+        </is>
+      </c>
+      <c r="F3" s="7" t="inlineStr">
+        <is>
+          <t>match_id</t>
+        </is>
+      </c>
+      <c r="G3" s="7" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H3" s="7" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I3" s="7" t="inlineStr">
+        <is>
+          <t>_dlt_parent_id is only the join key: LEFT JOIN to stg_matches__matches on matches__players._dlt_parent_id = matches.dlt_row_id, then take source_match_id from that match row</t>
+        </is>
+      </c>
+      <c r="J3" s="7" t="inlineStr">
+        <is>
+          <t>_dlt_parent_id doesn't turn into this column, it's how we find the parent match and pick up its match_id. LEFT JOIN, not INNER, so an orphaned player row shows up as a NULL instead of vanishing</t>
+        </is>
+      </c>
+      <c r="K3" s="7" t="inlineStr">
+        <is>
+          <t>not_null, relationships: raw matches__players._dlt_parent_id -&gt; matches._dlt_id (lives in the source yml, 0 orphans today). it points at the parent row's dlt id, not match_id, because match_id repeats. after the LEFT JOIN, not_null on source_match_id catches any orphan — (singular) exactly 10 rows per _dlt_parent_id (every match is 5v5), tests/singular/assert_ten_players_per_match.sql</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="29" customHeight="1">
+      <c r="A4" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_players</t>
+        </is>
+      </c>
+      <c r="B4" s="6" t="inlineStr">
+        <is>
+          <t>account_id</t>
+        </is>
+      </c>
+      <c r="C4" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D4" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E4" s="6" t="inlineStr">
+        <is>
           <t>matches__players</t>
         </is>
       </c>
-      <c r="F3" s="7" t="inlineStr">
-        <is>
-          <t>_dlt_parent_id</t>
-        </is>
-      </c>
-      <c r="G3" s="7" t="inlineStr">
-        <is>
-          <t>TEXT</t>
-        </is>
-      </c>
-      <c r="H3" s="7" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I3" s="7" t="inlineStr">
-        <is>
-          <t>LEFT JOIN to stg_opendota__matches on _dlt_parent_id = matches.dlt_row_id, return matches.source_match_id</t>
-        </is>
-      </c>
-      <c r="J3" s="7" t="inlineStr">
-        <is>
-          <t>has to be a LEFT JOIN, same reasoning as everywhere else — an orphaned player row shouldn't just vanish</t>
-        </is>
-      </c>
-      <c r="K3" s="7" t="inlineStr"/>
-    </row>
-    <row r="4">
-      <c r="A4" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_players</t>
-        </is>
-      </c>
-      <c r="B4" s="6" t="inlineStr">
+      <c r="F4" s="6" t="inlineStr">
         <is>
           <t>account_id</t>
         </is>
       </c>
-      <c r="C4" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D4" s="6" t="inlineStr">
+      <c r="G4" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H4" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="E4" s="6" t="inlineStr">
+      <c r="I4" s="6" t="inlineStr">
+        <is>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J4" s="6" t="inlineStr">
+        <is>
+          <t>genuinely nullable — 709 of 1740 rows populated (about 41%), missing for private profiles</t>
+        </is>
+      </c>
+      <c r="K4" s="6" t="inlineStr">
+        <is>
+          <t>none — nullable by nature (private profiles), so no not_null</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="58" customHeight="1">
+      <c r="A5" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_players</t>
+        </is>
+      </c>
+      <c r="B5" s="6" t="inlineStr">
+        <is>
+          <t>rank_bracket_id</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>YES</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
         <is>
           <t>matches__players</t>
         </is>
       </c>
-      <c r="F4" s="6" t="inlineStr">
-        <is>
-          <t>account_id</t>
-        </is>
-      </c>
-      <c r="G4" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H4" s="6" t="inlineStr">
+      <c r="F5" s="6" t="inlineStr">
+        <is>
+          <t>rank_tier</t>
+        </is>
+      </c>
+      <c r="G5" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H5" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="I4" s="6" t="inlineStr">
-        <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J4" s="6" t="inlineStr">
-        <is>
-          <t>genuinely nullable — 604 of 1510 populated, missing for private profiles</t>
-        </is>
-      </c>
-      <c r="K4" s="6" t="inlineStr"/>
-    </row>
-    <row r="5">
-      <c r="A5" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_players</t>
-        </is>
-      </c>
-      <c r="B5" s="6" t="inlineStr">
-        <is>
-          <t>rank_bracket_id</t>
-        </is>
-      </c>
-      <c r="C5" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D5" s="6" t="inlineStr">
+      <c r="I5" s="6" t="inlineStr">
+        <is>
+          <t>floor(rank_tier / 10) — NULL stays NULL</t>
+        </is>
+      </c>
+      <c r="J5" s="6" t="inlineStr">
+        <is>
+          <t>joins to dim_rank_tier at mart. nullable — 566 of 1740 rows have a rank (about a third)</t>
+        </is>
+      </c>
+      <c r="K5" s="6" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=1, max_value=8) on the non-null values — the 8 medals, Herald to Immortal (1 to 8 today). no not_null, most players have no rank — also floor(rank_tier / 10) between 1 and 8, checked separately from the star digit (generic test, table-level dbt_utils.expression_is_true, source yml)</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="43.5" customHeight="1">
+      <c r="A6" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_players</t>
+        </is>
+      </c>
+      <c r="B6" s="6" t="inlineStr">
+        <is>
+          <t>rank_star</t>
+        </is>
+      </c>
+      <c r="C6" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D6" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="E5" s="6" t="inlineStr">
+      <c r="E6" s="6" t="inlineStr">
         <is>
           <t>matches__players</t>
         </is>
       </c>
-      <c r="F5" s="6" t="inlineStr">
+      <c r="F6" s="6" t="inlineStr">
         <is>
           <t>rank_tier</t>
         </is>
       </c>
-      <c r="G5" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H5" s="6" t="inlineStr">
+      <c r="G6" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H6" s="6" t="inlineStr">
         <is>
           <t>YES</t>
         </is>
       </c>
-      <c r="I5" s="6" t="inlineStr">
-        <is>
-          <t>floor(rank_tier / 10)</t>
-        </is>
-      </c>
-      <c r="J5" s="6" t="inlineStr">
-        <is>
-          <t>joins to dim_rank_tier at mart. nullable — 486 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K5" s="6" t="inlineStr"/>
-    </row>
-    <row r="6">
-      <c r="A6" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_players</t>
-        </is>
-      </c>
-      <c r="B6" s="6" t="inlineStr">
-        <is>
-          <t>rank_star</t>
-        </is>
-      </c>
-      <c r="C6" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D6" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="E6" s="6" t="inlineStr">
+      <c r="I6" s="6" t="inlineStr">
+        <is>
+          <t>mod(rank_tier, 10) — NULL stays NULL</t>
+        </is>
+      </c>
+      <c r="J6" s="6" t="inlineStr">
+        <is>
+          <t>nullable, same source as rank_bracket_id</t>
+        </is>
+      </c>
+      <c r="K6" s="6" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0, max_value=5) — 1 to 5 stars, and 0 shows up for Immortal (rank_tier 80). no not_null — also mod(rank_tier, 10) between 0 and 5, checked separately from the bracket digit (generic test, table-level dbt_utils.expression_is_true, source yml)</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" ht="101.5" customHeight="1">
+      <c r="A7" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_players</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>player_slot</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
         <is>
           <t>matches__players</t>
         </is>
       </c>
-      <c r="F6" s="6" t="inlineStr">
-        <is>
-          <t>rank_tier</t>
-        </is>
-      </c>
-      <c r="G6" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H6" s="6" t="inlineStr">
-        <is>
-          <t>YES</t>
-        </is>
-      </c>
-      <c r="I6" s="6" t="inlineStr">
-        <is>
-          <t>mod(rank_tier, 10)</t>
-        </is>
-      </c>
-      <c r="J6" s="6" t="inlineStr">
-        <is>
-          <t>nullable, same source as rank_bracket_id</t>
-        </is>
-      </c>
-      <c r="K6" s="6" t="inlineStr"/>
-    </row>
-    <row r="7">
-      <c r="A7" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_players</t>
-        </is>
-      </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="F7" s="6" t="inlineStr">
         <is>
           <t>player_slot</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D7" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E7" s="6" t="inlineStr">
+      <c r="G7" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H7" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I7" s="6" t="inlineStr">
+        <is>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J7" s="6" t="inlineStr">
+        <is>
+          <t>0-4 is Radiant, 128-132 is Dire</t>
+        </is>
+      </c>
+      <c r="K7" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_values: [0, 1, 2, 3, 4, 128, 129, 130, 131, 132] — fixed by the game's 10 slots, not something the API grows. also dbt_utils.unique_combination_of_columns on (_dlt_parent_id, player_slot) (generic test, source yml) — one player per slot per match, 0 duplicates today</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" ht="72.5" customHeight="1">
+      <c r="A8" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_players</t>
+        </is>
+      </c>
+      <c r="B8" s="6" t="inlineStr">
+        <is>
+          <t>source_hero_id</t>
+        </is>
+      </c>
+      <c r="C8" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="D8" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E8" s="6" t="inlineStr">
         <is>
           <t>matches__players</t>
         </is>
       </c>
-      <c r="F7" s="6" t="inlineStr">
-        <is>
-          <t>player_slot</t>
-        </is>
-      </c>
-      <c r="G7" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H7" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I7" s="6" t="inlineStr">
-        <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J7" s="6" t="inlineStr"/>
-      <c r="K7" s="6" t="inlineStr"/>
-    </row>
-    <row r="8">
-      <c r="A8" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_players</t>
-        </is>
-      </c>
-      <c r="B8" s="6" t="inlineStr">
-        <is>
-          <t>source_hero_id</t>
-        </is>
-      </c>
-      <c r="C8" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="D8" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E8" s="6" t="inlineStr">
+      <c r="F8" s="6" t="inlineStr">
+        <is>
+          <t>hero_id</t>
+        </is>
+      </c>
+      <c r="G8" s="6" t="inlineStr">
+        <is>
+          <t>NUMBER</t>
+        </is>
+      </c>
+      <c r="H8" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Rename hero_id -&gt; source_hero_id</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>hero_id 0 means no hero was picked — 50 rows today, all with level 0 and zero stats. keep them (raw immutability) and handle with an unknown-hero row at mart, same idea as the private-profile players</t>
+        </is>
+      </c>
+      <c r="K8" s="6" t="inlineStr">
+        <is>
+          <t>not_null, relationships: raw matches__players.hero_id -&gt; heroes.id (source yml) with a where of hero_id != 0, because those 50 no-hero rows would fail a plain check</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="43.5" customHeight="1">
+      <c r="A9" s="6" t="inlineStr">
+        <is>
+          <t>stg_matches__match_players</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>is_radiant</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>BOOLEAN</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>NO</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
         <is>
           <t>matches__players</t>
         </is>
       </c>
-      <c r="F8" s="6" t="inlineStr">
-        <is>
-          <t>hero_id</t>
-        </is>
-      </c>
-      <c r="G8" s="6" t="inlineStr">
-        <is>
-          <t>NUMBER</t>
-        </is>
-      </c>
-      <c r="H8" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="I8" s="6" t="inlineStr">
-        <is>
-          <t>Rename; joins to stg_opendota__heroes.source_hero_id</t>
-        </is>
-      </c>
-      <c r="J8" s="6" t="inlineStr"/>
-      <c r="K8" s="6" t="inlineStr"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="6" t="inlineStr">
-        <is>
-          <t>stg_opendota__match_players</t>
-        </is>
-      </c>
-      <c r="B9" s="6" t="inlineStr">
+      <c r="F9" s="6" t="inlineStr">
         <is>
           <t>is_radiant</t>
         </is>
       </c>
-      <c r="C9" s="6" t="inlineStr">
+      <c r="G9" s="6" t="inlineStr">
         <is>
           <t>BOOLEAN</t>
         </is>
       </c>
-      <c r="D9" s="6" t="inlineStr">
-        <is>
-          <t>NO</t>
-        </is>
-      </c>
-      <c r="E9" s="6" t="inlineStr">
-        <is>
-          <t>matches__players</t>
-        </is>
-      </c>
-      <c r="F9" s="6" t="inlineStr">
-        <is>
-          <t>is_radiant</t>
-        </is>
-      </c>
-      <c r="G9" s="6" t="inlineStr">
-        <is>
-          <t>BOOLEAN</t>
-        </is>
-      </c>
       <c r="H9" s="6" t="inlineStr">
         <is>
           <t>NO</t>
@@ -5227,16 +5321,24 @@
       </c>
       <c r="I9" s="6" t="inlineStr">
         <is>
-          <t>Cast boolean</t>
-        </is>
-      </c>
-      <c r="J9" s="6" t="inlineStr"/>
-      <c r="K9" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J9" s="6" t="inlineStr">
+        <is>
+          <t>always agrees with player_slot (slot under 128 = Radiant) — checked on all 1740 rows</t>
+        </is>
+      </c>
+      <c r="K9" s="6" t="inlineStr">
+        <is>
+          <t>not_null, plus a custom check that (player_slot &lt; 128) = is_radiant — holds for every row today, so it's a real invariant</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B10" s="6" t="inlineStr">
@@ -5276,16 +5378,20 @@
       </c>
       <c r="I10" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J10" s="6" t="inlineStr"/>
-      <c r="K10" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J10" s="6" t="n"/>
+      <c r="K10" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B11" s="6" t="inlineStr">
@@ -5325,16 +5431,20 @@
       </c>
       <c r="I11" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J11" s="6" t="inlineStr"/>
-      <c r="K11" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J11" s="6" t="n"/>
+      <c r="K11" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B12" s="6" t="inlineStr">
@@ -5374,16 +5484,20 @@
       </c>
       <c r="I12" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J12" s="6" t="inlineStr"/>
-      <c r="K12" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J12" s="6" t="n"/>
+      <c r="K12" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B13" s="6" t="inlineStr">
@@ -5423,21 +5537,25 @@
       </c>
       <c r="I13" s="6" t="inlineStr">
         <is>
-          <t>Cast numeric</t>
-        </is>
-      </c>
-      <c r="J13" s="6" t="inlineStr"/>
-      <c r="K13" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J13" s="6" t="n"/>
+      <c r="K13" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B14" s="6" t="inlineStr">
         <is>
-          <t>gold_per_minute</t>
+          <t>gold_per_min</t>
         </is>
       </c>
       <c r="C14" s="6" t="inlineStr">
@@ -5472,21 +5590,25 @@
       </c>
       <c r="I14" s="6" t="inlineStr">
         <is>
-          <t>Rename</t>
-        </is>
-      </c>
-      <c r="J14" s="6" t="inlineStr"/>
-      <c r="K14" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J14" s="6" t="n"/>
+      <c r="K14" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B15" s="6" t="inlineStr">
         <is>
-          <t>xp_per_minute</t>
+          <t>xp_per_min</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
@@ -5521,16 +5643,20 @@
       </c>
       <c r="I15" s="6" t="inlineStr">
         <is>
-          <t>Rename</t>
-        </is>
-      </c>
-      <c r="J15" s="6" t="inlineStr"/>
-      <c r="K15" s="6" t="inlineStr"/>
-    </row>
-    <row r="16">
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J15" s="6" t="n"/>
+      <c r="K15" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="43.5" customHeight="1">
       <c r="A16" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B16" s="6" t="inlineStr">
@@ -5570,16 +5696,24 @@
       </c>
       <c r="I16" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J16" s="6" t="inlineStr"/>
-      <c r="K16" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J16" s="6" t="inlineStr">
+        <is>
+          <t>0 is real here — it's the 50 no-hero rows</t>
+        </is>
+      </c>
+      <c r="K16" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0) — max is 30 today but the level cap has moved between patches before, so no upper cap</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B17" s="6" t="inlineStr">
@@ -5619,16 +5753,20 @@
       </c>
       <c r="I17" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J17" s="6" t="inlineStr"/>
-      <c r="K17" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J17" s="6" t="n"/>
+      <c r="K17" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B18" s="6" t="inlineStr">
@@ -5668,16 +5806,20 @@
       </c>
       <c r="I18" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J18" s="6" t="inlineStr"/>
-      <c r="K18" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J18" s="6" t="n"/>
+      <c r="K18" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B19" s="6" t="inlineStr">
@@ -5717,16 +5859,20 @@
       </c>
       <c r="I19" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J19" s="6" t="inlineStr"/>
-      <c r="K19" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J19" s="6" t="n"/>
+      <c r="K19" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B20" s="6" t="inlineStr">
@@ -5766,16 +5912,20 @@
       </c>
       <c r="I20" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J20" s="6" t="inlineStr"/>
-      <c r="K20" s="6" t="inlineStr"/>
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J20" s="6" t="n"/>
+      <c r="K20" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B21" s="6" t="inlineStr">
@@ -5815,16 +5965,20 @@
       </c>
       <c r="I21" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
-        </is>
-      </c>
-      <c r="J21" s="6" t="inlineStr"/>
-      <c r="K21" s="6" t="inlineStr"/>
-    </row>
-    <row r="22">
+          <t>Keep as-is</t>
+        </is>
+      </c>
+      <c r="J21" s="6" t="n"/>
+      <c r="K21" s="6" t="inlineStr">
+        <is>
+          <t>not_null, accepted_range(min_value=0)</t>
+        </is>
+      </c>
+    </row>
+    <row r="22" ht="43.5" customHeight="1">
       <c r="A22" s="8" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B22" s="8" t="inlineStr">
@@ -5864,20 +6018,24 @@
       </c>
       <c r="I22" s="8" t="inlineStr">
         <is>
-          <t>Cast numeric (0-1)</t>
+          <t>Keep as-is</t>
         </is>
       </c>
       <c r="J22" s="8" t="inlineStr">
         <is>
-          <t>keeping for now, revisit later — parser-dependent, only 50 of 1510 populated right now</t>
-        </is>
-      </c>
-      <c r="K22" s="8" t="inlineStr"/>
-    </row>
-    <row r="23">
+          <t>keeping for now, revisit later — parser-dependent, only 70 of 1740 rows (4%) populated right now</t>
+        </is>
+      </c>
+      <c r="K22" s="8" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0, max_value=1) on the non-null values (0 to 1 today). no not_null — only parsed matches have it</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="29" customHeight="1">
       <c r="A23" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B23" s="6" t="inlineStr">
@@ -5917,20 +6075,24 @@
       </c>
       <c r="I23" s="6" t="inlineStr">
         <is>
-          <t>Cast integer</t>
+          <t>Keep as-is</t>
         </is>
       </c>
       <c r="J23" s="6" t="inlineStr">
         <is>
-          <t>parser-dependent, only 50 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K23" s="6" t="inlineStr"/>
-    </row>
-    <row r="24">
+          <t>parser-dependent, only 70 of 1740 populated</t>
+        </is>
+      </c>
+      <c r="K23" s="6" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0), no not_null — parser-dependent</t>
+        </is>
+      </c>
+    </row>
+    <row r="24" ht="43.5" customHeight="1">
       <c r="A24" s="8" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B24" s="8" t="inlineStr">
@@ -5970,20 +6132,24 @@
       </c>
       <c r="I24" s="8" t="inlineStr">
         <is>
-          <t>Cast integer</t>
+          <t>Keep as-is</t>
         </is>
       </c>
       <c r="J24" s="8" t="inlineStr">
         <is>
-          <t>keeping for now, revisit later — parser-dependent, only 50 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K24" s="8" t="inlineStr"/>
-    </row>
-    <row r="25">
+          <t>keeping for now, revisit later — parser-dependent, only 70 of 1740 populated (and every value is 0 so far)</t>
+        </is>
+      </c>
+      <c r="K24" s="8" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0), no not_null — parser-dependent</t>
+        </is>
+      </c>
+    </row>
+    <row r="25" ht="29" customHeight="1">
       <c r="A25" s="8" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B25" s="8" t="inlineStr">
@@ -6023,20 +6189,24 @@
       </c>
       <c r="I25" s="8" t="inlineStr">
         <is>
-          <t>Keep raw code; decode at mart</t>
+          <t>Keep as-is — raw code, decode at mart</t>
         </is>
       </c>
       <c r="J25" s="8" t="inlineStr">
         <is>
-          <t>keeping for now, revisit later — parser-dependent, only 50 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K25" s="8" t="inlineStr"/>
-    </row>
-    <row r="26">
+          <t>keeping for now, revisit later — parser-dependent, only 70 of 1740 populated. codes 1 to 3 so far</t>
+        </is>
+      </c>
+      <c r="K25" s="8" t="inlineStr">
+        <is>
+          <t>none — raw API code so no accepted_values, parser-dependent so no not_null</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="29" customHeight="1">
       <c r="A26" s="8" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B26" s="8" t="inlineStr">
@@ -6076,20 +6246,24 @@
       </c>
       <c r="I26" s="8" t="inlineStr">
         <is>
-          <t>Keep raw code; decode at mart</t>
+          <t>Keep as-is — raw code, decode at mart</t>
         </is>
       </c>
       <c r="J26" s="8" t="inlineStr">
         <is>
-          <t>keeping for now, revisit later — parser-dependent, only 50 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K26" s="8" t="inlineStr"/>
-    </row>
-    <row r="27">
+          <t>keeping for now, revisit later — parser-dependent, only 70 of 1740 populated. codes 1 to 3 so far</t>
+        </is>
+      </c>
+      <c r="K26" s="8" t="inlineStr">
+        <is>
+          <t>none — raw API code so no accepted_values, parser-dependent so no not_null</t>
+        </is>
+      </c>
+    </row>
+    <row r="27" ht="43.5" customHeight="1">
       <c r="A27" s="8" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B27" s="8" t="inlineStr">
@@ -6129,25 +6303,29 @@
       </c>
       <c r="I27" s="8" t="inlineStr">
         <is>
-          <t>Cast numeric</t>
+          <t>Keep as-is</t>
         </is>
       </c>
       <c r="J27" s="8" t="inlineStr">
         <is>
-          <t>keeping for now, revisit later — parser-dependent, only 50 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K27" s="8" t="inlineStr"/>
-    </row>
-    <row r="28">
+          <t>keeping for now, revisit later — parser-dependent, only 70 of 1740 populated. not a 0 to 1 ratio, it runs about 0.3 to 4.3</t>
+        </is>
+      </c>
+      <c r="K27" s="8" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0), no not_null — parser-dependent. don't cap it at 1</t>
+        </is>
+      </c>
+    </row>
+    <row r="28" ht="29" customHeight="1">
       <c r="A28" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B28" s="6" t="inlineStr">
         <is>
-          <t>actions_per_minute</t>
+          <t>actions_per_min</t>
         </is>
       </c>
       <c r="C28" s="6" t="inlineStr">
@@ -6182,20 +6360,24 @@
       </c>
       <c r="I28" s="6" t="inlineStr">
         <is>
-          <t>Rename</t>
+          <t>Keep as-is</t>
         </is>
       </c>
       <c r="J28" s="6" t="inlineStr">
         <is>
-          <t>parser-dependent, only 50 of 1510 populated</t>
-        </is>
-      </c>
-      <c r="K28" s="6" t="inlineStr"/>
+          <t>parser-dependent, only 70 of 1740 populated</t>
+        </is>
+      </c>
+      <c r="K28" s="6" t="inlineStr">
+        <is>
+          <t>accepted_range(min_value=0), no not_null — parser-dependent</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" s="6" t="inlineStr">
         <is>
-          <t>stg_opendota__match_players</t>
+          <t>stg_matches__match_players</t>
         </is>
       </c>
       <c r="B29" s="6" t="inlineStr">
@@ -6235,11 +6417,15 @@
       </c>
       <c r="I29" s="6" t="inlineStr">
         <is>
-          <t>Rename, lineage only</t>
-        </is>
-      </c>
-      <c r="J29" s="6" t="inlineStr"/>
-      <c r="K29" s="6" t="inlineStr"/>
+          <t>Rename _dlt_id -&gt; dlt_row_id</t>
+        </is>
+      </c>
+      <c r="J29" s="6" t="n"/>
+      <c r="K29" s="6" t="inlineStr">
+        <is>
+          <t>not_null, unique</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <autoFilter ref="A1:K29"/>

</xml_diff>

<commit_message>
docs: update sttm staging to mart
</commit_message>
<xml_diff>
--- a/docs/sttm_raw_to_staging.xlsx
+++ b/docs/sttm_raw_to_staging.xlsx
@@ -92,7 +92,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="3">
     <border>
       <left/>
       <right/>
@@ -115,11 +115,25 @@
       </bottom>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color rgb="FFD0D0D0"/>
+      </left>
+      <right style="thin">
+        <color rgb="FFD0D0D0"/>
+      </right>
+      <top style="thin">
+        <color rgb="FFD0D0D0"/>
+      </top>
+      <bottom style="thin">
+        <color rgb="FFD0D0D0"/>
+      </bottom>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
@@ -143,6 +157,9 @@
       <alignment vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="2" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -2045,7 +2062,11 @@
           <t>Rename id -&gt; source_game_mode_id</t>
         </is>
       </c>
-      <c r="J3" s="6" t="n"/>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>unlike region, constants_game_mode loaded correctly as a proper array with numeric ids intact from the start — it never hit the dict-key ingestion issue that left region's id as TEXT, so no cast is needed here at all.</t>
+        </is>
+      </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>
@@ -2459,7 +2480,11 @@
           <t>Rename id -&gt; source_lobby_type_id</t>
         </is>
       </c>
-      <c r="J3" s="6" t="n"/>
+      <c r="J3" s="9" t="inlineStr">
+        <is>
+          <t>unlike region, constants_lobby_type loaded correctly as a proper array with numeric ids intact from the start — it never hit the dict-key ingestion issue that left region's id as TEXT, so no cast is needed here at all.</t>
+        </is>
+      </c>
       <c r="K3" s="6" t="inlineStr">
         <is>
           <t>not_null, unique</t>

</xml_diff>